<commit_message>
Refine q2784 Helm migration delivery
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R57fd6bae79a5451b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R1ee9d872a84a4cc4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
         <x:v>目标输出文件</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>output/chart、output/values、output/renders、output/reports、output/tools、output/RELEASE-NOTES.md和output/README.txt</x:v>
+        <x:v>output/chart、output/values、output/renders、output/reports、output/RELEASE-NOTES.md和output/README.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -407,10 +407,10 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="5" t="str">
-        <x:v>岗位接续</x:v>
+        <x:v>维护窗安排</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
-        <x:v>观测团队核对对象清单，维护窗值班负责现场应用与仪表盘观察</x:v>
+        <x:v>只影响租户仪表盘标题和查询；依次处理development和production，每个环境观察15分钟，异常时使用starter中的旧Chart</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -426,7 +426,7 @@
         <x:v>可验证点</x:v>
       </x:c>
       <x:c r="B19" s="5" t="str">
-        <x:v>输入消费者、values字段集合、schema约束、tpl调用数、对象集合、标题与查询、报告业务键和岗位边界</x:v>
+        <x:v>输入消费者、values字段集合、schema约束、tpl调用数、对象集合、标题与查询、报告业务键和维护窗安排</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">

</xml_diff>